<commit_message>
Atualização automática diária da base
</commit_message>
<xml_diff>
--- a/base_despesas/2026/despesas_202609.xlsx
+++ b/base_despesas/2026/despesas_202609.xlsx
@@ -734,7 +734,7 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="AJ34" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="AJ35" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="AJ36" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="AJ37" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="AJ38" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="AJ39" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6054,7 +6054,7 @@
       </c>
       <c r="AJ40" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="AJ41" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="AJ42" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="AJ43" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="AJ44" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="AJ45" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -6894,7 +6894,7 @@
       </c>
       <c r="AJ46" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AJ47" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="AJ48" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7454,7 @@
       </c>
       <c r="AJ50" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="AJ51" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="AJ52" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AJ53" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="AJ54" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="AJ55" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="AJ56" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="AJ57" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="AJ58" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="AJ59" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8854,7 +8854,7 @@
       </c>
       <c r="AJ60" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="AJ61" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AJ62" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9274,7 +9274,7 @@
       </c>
       <c r="AJ63" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="AJ64" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AJ65" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="AJ66" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9834,7 +9834,7 @@
       </c>
       <c r="AJ67" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -9974,7 +9974,7 @@
       </c>
       <c r="AJ68" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10114,7 +10114,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10394,7 +10394,7 @@
       </c>
       <c r="AJ71" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10534,7 +10534,7 @@
       </c>
       <c r="AJ72" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10674,7 +10674,7 @@
       </c>
       <c r="AJ73" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10814,7 +10814,7 @@
       </c>
       <c r="AJ74" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -10954,7 +10954,7 @@
       </c>
       <c r="AJ75" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11094,7 @@
       </c>
       <c r="AJ76" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11234,7 +11234,7 @@
       </c>
       <c r="AJ77" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11374,7 +11374,7 @@
       </c>
       <c r="AJ78" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11514,7 +11514,7 @@
       </c>
       <c r="AJ79" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11654,7 +11654,7 @@
       </c>
       <c r="AJ80" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11794,7 +11794,7 @@
       </c>
       <c r="AJ81" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -11934,7 +11934,7 @@
       </c>
       <c r="AJ82" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="AJ83" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12214,7 @@
       </c>
       <c r="AJ84" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12354,7 +12354,7 @@
       </c>
       <c r="AJ85" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12494,7 +12494,7 @@
       </c>
       <c r="AJ86" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12634,7 +12634,7 @@
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12774,7 +12774,7 @@
       </c>
       <c r="AJ88" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -12914,7 +12914,7 @@
       </c>
       <c r="AJ89" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13054,7 +13054,7 @@
       </c>
       <c r="AJ90" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13194,7 +13194,7 @@
       </c>
       <c r="AJ91" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="AJ92" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13474,7 +13474,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="AJ94" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -13894,7 +13894,7 @@
       </c>
       <c r="AJ96" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="AJ97" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14174,7 +14174,7 @@
       </c>
       <c r="AJ98" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14314,7 +14314,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14594,7 +14594,7 @@
       </c>
       <c r="AJ101" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14734,7 +14734,7 @@
       </c>
       <c r="AJ102" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -14874,7 +14874,7 @@
       </c>
       <c r="AJ103" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15014,7 +15014,7 @@
       </c>
       <c r="AJ104" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15154,7 +15154,7 @@
       </c>
       <c r="AJ105" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15294,7 +15294,7 @@
       </c>
       <c r="AJ106" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15434,7 +15434,7 @@
       </c>
       <c r="AJ107" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15574,7 +15574,7 @@
       </c>
       <c r="AJ108" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15714,7 +15714,7 @@
       </c>
       <c r="AJ109" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15854,7 +15854,7 @@
       </c>
       <c r="AJ110" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -15994,7 +15994,7 @@
       </c>
       <c r="AJ111" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16134,7 +16134,7 @@
       </c>
       <c r="AJ112" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16274,7 +16274,7 @@
       </c>
       <c r="AJ113" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16414,7 +16414,7 @@
       </c>
       <c r="AJ114" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16554,7 +16554,7 @@
       </c>
       <c r="AJ115" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16694,7 +16694,7 @@
       </c>
       <c r="AJ116" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16834,7 +16834,7 @@
       </c>
       <c r="AJ117" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -16974,7 +16974,7 @@
       </c>
       <c r="AJ118" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17114,7 +17114,7 @@
       </c>
       <c r="AJ119" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17254,7 +17254,7 @@
       </c>
       <c r="AJ120" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17394,7 +17394,7 @@
       </c>
       <c r="AJ121" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17534,7 +17534,7 @@
       </c>
       <c r="AJ122" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17674,7 +17674,7 @@
       </c>
       <c r="AJ123" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17814,7 +17814,7 @@
       </c>
       <c r="AJ124" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -17954,7 +17954,7 @@
       </c>
       <c r="AJ125" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18094,7 +18094,7 @@
       </c>
       <c r="AJ126" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18234,7 +18234,7 @@
       </c>
       <c r="AJ127" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18374,7 +18374,7 @@
       </c>
       <c r="AJ128" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18514,7 +18514,7 @@
       </c>
       <c r="AJ129" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18654,7 +18654,7 @@
       </c>
       <c r="AJ130" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18794,7 +18794,7 @@
       </c>
       <c r="AJ131" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -18934,7 +18934,7 @@
       </c>
       <c r="AJ132" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19074,7 +19074,7 @@
       </c>
       <c r="AJ133" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19214,7 +19214,7 @@
       </c>
       <c r="AJ134" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19354,7 +19354,7 @@
       </c>
       <c r="AJ135" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       </c>
       <c r="AJ136" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19634,7 +19634,7 @@
       </c>
       <c r="AJ137" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="AJ138" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
       </c>
       <c r="AJ139" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20054,7 +20054,7 @@
       </c>
       <c r="AJ140" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20194,7 +20194,7 @@
       </c>
       <c r="AJ141" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20334,7 +20334,7 @@
       </c>
       <c r="AJ142" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20474,7 +20474,7 @@
       </c>
       <c r="AJ143" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20614,7 +20614,7 @@
       </c>
       <c r="AJ144" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20754,7 +20754,7 @@
       </c>
       <c r="AJ145" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -20894,7 +20894,7 @@
       </c>
       <c r="AJ146" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21034,7 +21034,7 @@
       </c>
       <c r="AJ147" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21174,7 +21174,7 @@
       </c>
       <c r="AJ148" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="AJ149" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       </c>
       <c r="AJ150" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21594,7 +21594,7 @@
       </c>
       <c r="AJ151" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21734,7 +21734,7 @@
       </c>
       <c r="AJ152" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -21874,7 +21874,7 @@
       </c>
       <c r="AJ153" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22014,7 +22014,7 @@
       </c>
       <c r="AJ154" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22154,7 +22154,7 @@
       </c>
       <c r="AJ155" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22294,7 +22294,7 @@
       </c>
       <c r="AJ156" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22434,7 +22434,7 @@
       </c>
       <c r="AJ157" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22574,7 +22574,7 @@
       </c>
       <c r="AJ158" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22714,7 +22714,7 @@
       </c>
       <c r="AJ159" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22854,7 +22854,7 @@
       </c>
       <c r="AJ160" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -22994,7 +22994,7 @@
       </c>
       <c r="AJ161" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23134,7 +23134,7 @@
       </c>
       <c r="AJ162" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23274,7 +23274,7 @@
       </c>
       <c r="AJ163" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23414,7 +23414,7 @@
       </c>
       <c r="AJ164" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23554,7 +23554,7 @@
       </c>
       <c r="AJ165" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23694,7 +23694,7 @@
       </c>
       <c r="AJ166" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23834,7 +23834,7 @@
       </c>
       <c r="AJ167" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -23974,7 +23974,7 @@
       </c>
       <c r="AJ168" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24114,7 +24114,7 @@
       </c>
       <c r="AJ169" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24254,7 +24254,7 @@
       </c>
       <c r="AJ170" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24394,7 +24394,7 @@
       </c>
       <c r="AJ171" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24534,7 +24534,7 @@
       </c>
       <c r="AJ172" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24674,7 +24674,7 @@
       </c>
       <c r="AJ173" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24814,7 +24814,7 @@
       </c>
       <c r="AJ174" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -24954,7 +24954,7 @@
       </c>
       <c r="AJ175" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25094,7 +25094,7 @@
       </c>
       <c r="AJ176" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25234,7 +25234,7 @@
       </c>
       <c r="AJ177" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25374,7 +25374,7 @@
       </c>
       <c r="AJ178" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25514,7 +25514,7 @@
       </c>
       <c r="AJ179" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25654,7 +25654,7 @@
       </c>
       <c r="AJ180" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25794,7 +25794,7 @@
       </c>
       <c r="AJ181" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -25934,7 +25934,7 @@
       </c>
       <c r="AJ182" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26074,7 +26074,7 @@
       </c>
       <c r="AJ183" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26214,7 +26214,7 @@
       </c>
       <c r="AJ184" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26354,7 +26354,7 @@
       </c>
       <c r="AJ185" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26494,7 +26494,7 @@
       </c>
       <c r="AJ186" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26634,7 +26634,7 @@
       </c>
       <c r="AJ187" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26774,7 +26774,7 @@
       </c>
       <c r="AJ188" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -26914,7 +26914,7 @@
       </c>
       <c r="AJ189" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27054,7 +27054,7 @@
       </c>
       <c r="AJ190" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27194,7 +27194,7 @@
       </c>
       <c r="AJ191" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27334,7 +27334,7 @@
       </c>
       <c r="AJ192" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27474,7 +27474,7 @@
       </c>
       <c r="AJ193" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27614,7 +27614,7 @@
       </c>
       <c r="AJ194" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27754,7 +27754,7 @@
       </c>
       <c r="AJ195" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -27894,7 +27894,7 @@
       </c>
       <c r="AJ196" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28034,7 +28034,7 @@
       </c>
       <c r="AJ197" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28174,7 +28174,7 @@
       </c>
       <c r="AJ198" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28314,7 +28314,7 @@
       </c>
       <c r="AJ199" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28454,7 +28454,7 @@
       </c>
       <c r="AJ200" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28594,7 +28594,7 @@
       </c>
       <c r="AJ201" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="AJ202" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -28874,7 +28874,7 @@
       </c>
       <c r="AJ203" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29014,7 +29014,7 @@
       </c>
       <c r="AJ204" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29154,7 +29154,7 @@
       </c>
       <c r="AJ205" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29294,7 +29294,7 @@
       </c>
       <c r="AJ206" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29434,7 +29434,7 @@
       </c>
       <c r="AJ207" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29574,7 +29574,7 @@
       </c>
       <c r="AJ208" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29714,7 +29714,7 @@
       </c>
       <c r="AJ209" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29854,7 +29854,7 @@
       </c>
       <c r="AJ210" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -29994,7 +29994,7 @@
       </c>
       <c r="AJ211" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30134,7 +30134,7 @@
       </c>
       <c r="AJ212" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30274,7 +30274,7 @@
       </c>
       <c r="AJ213" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30414,7 +30414,7 @@
       </c>
       <c r="AJ214" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30554,7 +30554,7 @@
       </c>
       <c r="AJ215" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30694,7 +30694,7 @@
       </c>
       <c r="AJ216" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30834,7 +30834,7 @@
       </c>
       <c r="AJ217" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -30974,7 +30974,7 @@
       </c>
       <c r="AJ218" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31114,7 +31114,7 @@
       </c>
       <c r="AJ219" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31254,7 +31254,7 @@
       </c>
       <c r="AJ220" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31394,7 +31394,7 @@
       </c>
       <c r="AJ221" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31534,7 +31534,7 @@
       </c>
       <c r="AJ222" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31674,7 +31674,7 @@
       </c>
       <c r="AJ223" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31814,7 +31814,7 @@
       </c>
       <c r="AJ224" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -31954,7 +31954,7 @@
       </c>
       <c r="AJ225" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>
@@ -32094,7 +32094,7 @@
       </c>
       <c r="AJ226" t="inlineStr">
         <is>
-          <t>06/09/2026 09:57:33</t>
+          <t>07/09/2026 12:13:15</t>
         </is>
       </c>
     </row>

</xml_diff>